<commit_message>
Redo bài6 and bài7 keeping the original workbook structure
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HiyVPr15dFfxwtDW3Tiv76
</commit_message>
<xml_diff>
--- a/excel_bai_tap/TranGiaHy_11a2_bài6.xlsx
+++ b/excel_bai_tap/TranGiaHy_11a2_bài6.xlsx
@@ -3,13 +3,15 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="24000" windowHeight="9300" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="24000" windowHeight="9300" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="bai 1" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2016" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2015" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2014" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Yeu cau" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Question" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="bai 1" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2016" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2015" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2014" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="DATA">'2016'!$C$3:$H$9</definedName>
@@ -625,6 +627,126 @@
 </styleSheet>
 </file>
 
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <twoCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>465896</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <to>
+      <col>12</col>
+      <colOff>55079</colOff>
+      <row>3</row>
+      <rowOff>5763</rowOff>
+    </to>
+    <grpSp>
+      <nvGrpSpPr>
+        <cNvPr id="3" name="Group 2"/>
+        <cNvGrpSpPr/>
+      </nvGrpSpPr>
+      <grpSpPr>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0">
+          <a:off x="1087092" y="0"/>
+          <a:ext cx="5718313" cy="651806"/>
+          <a:chOff x="10002807" y="3305175"/>
+          <a:chExt cx="9771093" cy="832807"/>
+        </a:xfrm>
+      </grpSpPr>
+      <pic>
+        <nvPicPr>
+          <cNvPr id="7" name="Picture 6"/>
+          <cNvPicPr>
+            <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+          </cNvPicPr>
+        </nvPicPr>
+        <blipFill>
+          <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+          <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:fillRect/>
+          </a:stretch>
+        </blipFill>
+        <spPr>
+          <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:off x="10358294" y="3459262"/>
+            <a:ext cx="1123949" cy="621523"/>
+          </a:xfrm>
+          <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
+            <avLst/>
+          </a:prstGeom>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:prstDash val="solid"/>
+          </a:ln>
+        </spPr>
+      </pic>
+    </grpSp>
+    <clientData/>
+  </twoCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <twoCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>143511</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <to>
+      <col>13</col>
+      <colOff>343743</colOff>
+      <row>2</row>
+      <rowOff>184462</rowOff>
+    </to>
+    <grpSp>
+      <nvGrpSpPr>
+        <cNvPr id="2" name="Group 1"/>
+        <cNvGrpSpPr/>
+      </nvGrpSpPr>
+      <grpSpPr>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0">
+          <a:off x="1970579" y="0"/>
+          <a:ext cx="5655459" cy="634735"/>
+          <a:chOff x="10002807" y="3305175"/>
+          <a:chExt cx="9744851" cy="809625"/>
+        </a:xfrm>
+      </grpSpPr>
+      <pic>
+        <nvPicPr>
+          <cNvPr id="6" name="Picture 5"/>
+          <cNvPicPr>
+            <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+          </cNvPicPr>
+        </nvPicPr>
+        <blipFill>
+          <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+          <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:fillRect/>
+          </a:stretch>
+        </blipFill>
+        <spPr>
+          <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:off x="10358292" y="3459263"/>
+            <a:ext cx="1442521" cy="621523"/>
+          </a:xfrm>
+          <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
+            <avLst/>
+          </a:prstGeom>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:prstDash val="solid"/>
+          </a:ln>
+        </spPr>
+      </pic>
+    </grpSp>
+    <clientData/>
+  </twoCellAnchor>
+</wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -911,6 +1033,1039 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A2:J26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15.75"/>
+  <cols>
+    <col width="4.7109375" customWidth="1" style="28" min="1" max="1"/>
+    <col width="4.5703125" customWidth="1" style="28" min="2" max="2"/>
+    <col width="9.140625" customWidth="1" style="28" min="3" max="16384"/>
+  </cols>
+  <sheetData>
+    <row r="2" ht="19.5" customHeight="1">
+      <c r="A2" s="62" t="inlineStr">
+        <is>
+          <t>Yêu cầu:</t>
+        </is>
+      </c>
+      <c r="B2" s="26" t="n"/>
+      <c r="C2" s="26" t="n"/>
+      <c r="D2" s="26" t="n"/>
+      <c r="E2" s="26" t="n"/>
+      <c r="F2" s="26" t="n"/>
+      <c r="G2" s="26" t="n"/>
+      <c r="H2" s="26" t="n"/>
+      <c r="I2" s="26" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="29" t="n"/>
+      <c r="B3" s="26" t="n"/>
+      <c r="C3" s="26" t="n"/>
+      <c r="D3" s="26" t="n"/>
+      <c r="E3" s="26" t="n"/>
+      <c r="F3" s="26" t="n"/>
+      <c r="G3" s="26" t="n"/>
+      <c r="H3" s="26" t="n"/>
+      <c r="I3" s="26" t="n"/>
+    </row>
+    <row r="4" ht="21.75" customHeight="1">
+      <c r="A4" s="29" t="n"/>
+      <c r="B4" s="26" t="inlineStr">
+        <is>
+          <t>Tạo thư mục &lt;HOTEN_MSSV&gt; để lưu các tập tin, nén thư mục này và nộp lên hệ thống Elearning</t>
+        </is>
+      </c>
+      <c r="C4" s="26" t="n"/>
+      <c r="D4" s="26" t="n"/>
+      <c r="E4" s="26" t="n"/>
+      <c r="F4" s="26" t="n"/>
+      <c r="G4" s="26" t="n"/>
+      <c r="H4" s="26" t="n"/>
+      <c r="I4" s="26" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="26" t="n"/>
+      <c r="B5" s="25" t="inlineStr">
+        <is>
+          <t>Chỉ thực hiện các yêu cầu trong trang tính này. Các trang tính khác dùng để hỗ trợ.</t>
+        </is>
+      </c>
+      <c r="C5" s="26" t="n"/>
+      <c r="D5" s="26" t="n"/>
+      <c r="E5" s="26" t="n"/>
+      <c r="F5" s="26" t="n"/>
+      <c r="G5" s="26" t="n"/>
+      <c r="H5" s="26" t="n"/>
+      <c r="I5" s="26" t="n"/>
+    </row>
+    <row r="6" customFormat="1" s="78">
+      <c r="A6" s="73" t="inlineStr">
+        <is>
+          <t>I.-</t>
+        </is>
+      </c>
+      <c r="B6" s="77" t="inlineStr">
+        <is>
+          <t>Trong trang tính bai 1 thực hiện các yêu cầu sau:</t>
+        </is>
+      </c>
+      <c r="C6" s="75" t="n"/>
+      <c r="D6" s="75" t="n"/>
+      <c r="E6" s="75" t="n"/>
+      <c r="F6" s="75" t="n"/>
+      <c r="G6" s="75" t="n"/>
+      <c r="H6" s="75" t="n"/>
+      <c r="I6" s="75" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="27" t="n"/>
+      <c r="B7" s="27" t="inlineStr">
+        <is>
+          <t>1/</t>
+        </is>
+      </c>
+      <c r="C7" s="26" t="inlineStr">
+        <is>
+          <t>Điền số thứ tự cho các cột STT (A4:A10 và K4:K10) (autofill).</t>
+        </is>
+      </c>
+      <c r="D7" s="26" t="n"/>
+      <c r="E7" s="26" t="n"/>
+      <c r="F7" s="26" t="n"/>
+      <c r="G7" s="26" t="n"/>
+      <c r="H7" s="26" t="n"/>
+      <c r="I7" s="26" t="n"/>
+      <c r="J7" s="26" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="27" t="n"/>
+      <c r="B8" s="27" t="inlineStr">
+        <is>
+          <t>2/</t>
+        </is>
+      </c>
+      <c r="C8" s="26" t="inlineStr">
+        <is>
+          <t>Trị giá = Số lượng * Đơn giá.</t>
+        </is>
+      </c>
+      <c r="D8" s="26" t="n"/>
+      <c r="E8" s="26" t="n"/>
+      <c r="F8" s="26" t="n"/>
+      <c r="G8" s="26" t="n"/>
+      <c r="H8" s="26" t="n"/>
+      <c r="I8" s="26" t="n"/>
+      <c r="J8" s="26" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="27" t="n"/>
+      <c r="B9" s="27" t="inlineStr">
+        <is>
+          <t>3/</t>
+        </is>
+      </c>
+      <c r="C9" s="26" t="inlineStr">
+        <is>
+          <t>Thuế = Trị giá * 5%.</t>
+        </is>
+      </c>
+      <c r="D9" s="26" t="n"/>
+      <c r="E9" s="26" t="n"/>
+      <c r="F9" s="26" t="n"/>
+      <c r="G9" s="26" t="n"/>
+      <c r="H9" s="26" t="n"/>
+      <c r="I9" s="26" t="n"/>
+      <c r="J9" s="26" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="27" t="n"/>
+      <c r="B10" s="27" t="inlineStr">
+        <is>
+          <t>4/</t>
+        </is>
+      </c>
+      <c r="C10" s="26" t="inlineStr">
+        <is>
+          <t>Cước chuyên chở = Số lượng * 1500.</t>
+        </is>
+      </c>
+      <c r="D10" s="26" t="n"/>
+      <c r="E10" s="26" t="n"/>
+      <c r="F10" s="26" t="n"/>
+      <c r="G10" s="26" t="n"/>
+      <c r="H10" s="26" t="n"/>
+      <c r="I10" s="26" t="n"/>
+      <c r="J10" s="26" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="27" t="n"/>
+      <c r="B11" s="27" t="inlineStr">
+        <is>
+          <t>5/</t>
+        </is>
+      </c>
+      <c r="C11" s="26" t="inlineStr">
+        <is>
+          <t>Cộng USD = Trị giá + Thuế + Cước chuyên chở.</t>
+        </is>
+      </c>
+      <c r="D11" s="26" t="n"/>
+      <c r="E11" s="26" t="n"/>
+      <c r="F11" s="26" t="n"/>
+      <c r="G11" s="26" t="n"/>
+      <c r="H11" s="26" t="n"/>
+      <c r="I11" s="26" t="n"/>
+      <c r="J11" s="26" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="27" t="n"/>
+      <c r="B12" s="27" t="inlineStr">
+        <is>
+          <t>6/</t>
+        </is>
+      </c>
+      <c r="C12" s="26" t="inlineStr">
+        <is>
+          <t>Cộng VNĐ được qui đổi dựa vào cột Cộng USD và Tỉ giá..</t>
+        </is>
+      </c>
+      <c r="D12" s="26" t="n"/>
+      <c r="E12" s="26" t="n"/>
+      <c r="F12" s="26" t="n"/>
+      <c r="G12" s="26" t="n"/>
+      <c r="H12" s="26" t="n"/>
+      <c r="I12" s="26" t="n"/>
+      <c r="J12" s="26" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="27" t="n"/>
+      <c r="B13" s="27" t="inlineStr">
+        <is>
+          <t>7/</t>
+        </is>
+      </c>
+      <c r="C13" s="26" t="inlineStr">
+        <is>
+          <t>Tổng lợi nhuận THÁNG 1 của từng mặt hàng được tính bằng lợi nhuận tháng 1 trong các năm 2014, 2015 và 2016 của mặt hàng tương ứng.</t>
+        </is>
+      </c>
+      <c r="D13" s="26" t="n"/>
+      <c r="E13" s="26" t="n"/>
+      <c r="F13" s="26" t="n"/>
+      <c r="G13" s="26" t="n"/>
+      <c r="H13" s="26" t="n"/>
+      <c r="I13" s="26" t="n"/>
+      <c r="J13" s="26" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="27" t="n"/>
+      <c r="B14" s="27" t="inlineStr">
+        <is>
+          <t>8/</t>
+        </is>
+      </c>
+      <c r="C14" s="26" t="inlineStr">
+        <is>
+          <t>Sao chép công thức sao cho có thể xác định được tổng lợi nhuận của từng mặt hàng trong từng tháng của cả 3 năm.</t>
+        </is>
+      </c>
+      <c r="D14" s="26" t="n"/>
+      <c r="E14" s="26" t="n"/>
+      <c r="F14" s="26" t="n"/>
+      <c r="G14" s="26" t="n"/>
+      <c r="H14" s="26" t="n"/>
+      <c r="I14" s="26" t="n"/>
+      <c r="J14" s="26" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="27" t="n"/>
+      <c r="B15" s="27" t="inlineStr">
+        <is>
+          <t>9/</t>
+        </is>
+      </c>
+      <c r="C15" s="26" t="inlineStr">
+        <is>
+          <t>Tính tổng lợi nhuận cho từng tháng của tất cả các mặt hàng.</t>
+        </is>
+      </c>
+      <c r="D15" s="26" t="n"/>
+      <c r="E15" s="26" t="n"/>
+      <c r="F15" s="26" t="n"/>
+      <c r="G15" s="26" t="n"/>
+      <c r="H15" s="26" t="n"/>
+      <c r="I15" s="26" t="n"/>
+      <c r="J15" s="26" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="27" t="n"/>
+      <c r="B16" s="27" t="inlineStr">
+        <is>
+          <t>10/</t>
+        </is>
+      </c>
+      <c r="C16" s="26" t="inlineStr">
+        <is>
+          <t>Xác định giá trị lỗ lớn nhất của tất cả các mặt hàng trong tháng 1.</t>
+        </is>
+      </c>
+      <c r="D16" s="26" t="n"/>
+      <c r="E16" s="26" t="n"/>
+      <c r="F16" s="26" t="n"/>
+      <c r="G16" s="26" t="n"/>
+      <c r="H16" s="26" t="n"/>
+      <c r="I16" s="26" t="n"/>
+      <c r="J16" s="26" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="27" t="n"/>
+      <c r="B17" s="27" t="inlineStr">
+        <is>
+          <t>11/</t>
+        </is>
+      </c>
+      <c r="C17" s="26" t="inlineStr">
+        <is>
+          <t>Xác định giá trị lãi lớn nhất của tất cả các mặt hàng trong tháng 3.</t>
+        </is>
+      </c>
+      <c r="D17" s="26" t="n"/>
+      <c r="E17" s="26" t="n"/>
+      <c r="F17" s="26" t="n"/>
+      <c r="G17" s="26" t="n"/>
+      <c r="H17" s="26" t="n"/>
+      <c r="I17" s="26" t="n"/>
+      <c r="J17" s="26" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="27" t="n"/>
+      <c r="B18" s="27" t="inlineStr">
+        <is>
+          <t>12/</t>
+        </is>
+      </c>
+      <c r="C18" s="26" t="inlineStr">
+        <is>
+          <t>Xác định giá trị lợi nhuận trung bình của tất cả các mặt hàng trong tháng 5.</t>
+        </is>
+      </c>
+      <c r="D18" s="26" t="n"/>
+      <c r="E18" s="26" t="n"/>
+      <c r="F18" s="26" t="n"/>
+      <c r="G18" s="26" t="n"/>
+      <c r="H18" s="26" t="n"/>
+      <c r="I18" s="26" t="n"/>
+      <c r="J18" s="26" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="27" t="n"/>
+      <c r="B19" s="27" t="inlineStr">
+        <is>
+          <t>13/</t>
+        </is>
+      </c>
+      <c r="C19" s="26" t="inlineStr">
+        <is>
+          <t>Lưu tập tin.</t>
+        </is>
+      </c>
+      <c r="D19" s="26" t="n"/>
+      <c r="E19" s="26" t="n"/>
+      <c r="F19" s="26" t="n"/>
+      <c r="G19" s="26" t="n"/>
+      <c r="H19" s="26" t="n"/>
+      <c r="I19" s="26" t="n"/>
+      <c r="J19" s="26" t="n"/>
+    </row>
+    <row r="20" customFormat="1" s="78">
+      <c r="A20" s="73" t="inlineStr">
+        <is>
+          <t>II.-</t>
+        </is>
+      </c>
+      <c r="B20" s="77" t="inlineStr">
+        <is>
+          <t>Trong trang tính 2016 thực hiện các yêu cầu sau:</t>
+        </is>
+      </c>
+      <c r="C20" s="75" t="n"/>
+      <c r="D20" s="75" t="n"/>
+      <c r="E20" s="75" t="n"/>
+      <c r="F20" s="75" t="n"/>
+      <c r="G20" s="75" t="n"/>
+      <c r="H20" s="75" t="n"/>
+      <c r="I20" s="75" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="27" t="n"/>
+      <c r="B21" s="27" t="inlineStr">
+        <is>
+          <t>1/</t>
+        </is>
+      </c>
+      <c r="C21" s="26" t="inlineStr">
+        <is>
+          <t>Đặt tên cho khối ô C3:H9 là DATA.</t>
+        </is>
+      </c>
+      <c r="D21" s="26" t="n"/>
+      <c r="E21" s="26" t="n"/>
+      <c r="F21" s="26" t="n"/>
+      <c r="G21" s="26" t="n"/>
+      <c r="H21" s="26" t="n"/>
+      <c r="I21" s="26" t="n"/>
+      <c r="J21" s="26" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="27" t="n"/>
+      <c r="B22" s="27" t="inlineStr">
+        <is>
+          <t>2/</t>
+        </is>
+      </c>
+      <c r="C22" s="26" t="inlineStr">
+        <is>
+          <t>Sử dụng tên khối DATA, xác định tổng lợi nhuận của tất cả các mặt hàng trong tất cả các tháng.</t>
+        </is>
+      </c>
+      <c r="D22" s="26" t="n"/>
+      <c r="E22" s="26" t="n"/>
+      <c r="F22" s="26" t="n"/>
+      <c r="G22" s="26" t="n"/>
+      <c r="H22" s="26" t="n"/>
+      <c r="I22" s="26" t="n"/>
+      <c r="J22" s="26" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="27" t="n"/>
+      <c r="B23" s="27" t="inlineStr">
+        <is>
+          <t>3/</t>
+        </is>
+      </c>
+      <c r="C23" s="26" t="inlineStr">
+        <is>
+          <t>Sử dụng tên khối DATA, xác định giá trị lợi nhuận lớn nhất của tất cả các mặt hàng trong tất cả các tháng</t>
+        </is>
+      </c>
+      <c r="D23" s="26" t="n"/>
+      <c r="E23" s="26" t="n"/>
+      <c r="F23" s="26" t="n"/>
+      <c r="G23" s="26" t="n"/>
+      <c r="H23" s="26" t="n"/>
+      <c r="I23" s="26" t="n"/>
+      <c r="J23" s="26" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="27" t="n"/>
+      <c r="B24" s="27" t="inlineStr">
+        <is>
+          <t>4/</t>
+        </is>
+      </c>
+      <c r="C24" s="26" t="inlineStr">
+        <is>
+          <t>Sử dụng tên khối DATA, xác định giá trị lợi nhuận trung bình của tất cả các mặt hàng trong tất cả các tháng</t>
+        </is>
+      </c>
+      <c r="D24" s="26" t="n"/>
+      <c r="E24" s="26" t="n"/>
+      <c r="F24" s="26" t="n"/>
+      <c r="G24" s="26" t="n"/>
+      <c r="H24" s="26" t="n"/>
+      <c r="I24" s="26" t="n"/>
+      <c r="J24" s="26" t="n"/>
+    </row>
+    <row r="25">
+      <c r="B25" s="27" t="inlineStr">
+        <is>
+          <t>5/</t>
+        </is>
+      </c>
+      <c r="C25" s="26" t="inlineStr">
+        <is>
+          <t>Hiển thị các công thức thay vì giá trị của công thức.</t>
+        </is>
+      </c>
+      <c r="I25" s="31" t="n"/>
+    </row>
+    <row r="26">
+      <c r="B26" s="27" t="inlineStr">
+        <is>
+          <t>6/</t>
+        </is>
+      </c>
+      <c r="C26" s="26" t="inlineStr">
+        <is>
+          <t>Lưu tập tin.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A2:P31"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15.75"/>
+  <cols>
+    <col width="4.7109375" customWidth="1" style="60" min="1" max="1"/>
+    <col width="4.5703125" customWidth="1" style="60" min="2" max="2"/>
+    <col width="9.140625" customWidth="1" style="60" min="3" max="16384"/>
+  </cols>
+  <sheetData>
+    <row r="2" ht="19.5" customHeight="1">
+      <c r="A2" s="62" t="inlineStr">
+        <is>
+          <t>Requirements:</t>
+        </is>
+      </c>
+      <c r="B2" s="26" t="n"/>
+      <c r="C2" s="26" t="n"/>
+      <c r="D2" s="26" t="n"/>
+      <c r="E2" s="26" t="n"/>
+      <c r="F2" s="26" t="n"/>
+      <c r="G2" s="26" t="n"/>
+      <c r="H2" s="26" t="n"/>
+      <c r="I2" s="26" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="29" t="n"/>
+      <c r="B3" s="26" t="n"/>
+      <c r="C3" s="26" t="n"/>
+      <c r="D3" s="26" t="n"/>
+      <c r="E3" s="26" t="n"/>
+      <c r="F3" s="26" t="n"/>
+      <c r="G3" s="26" t="n"/>
+      <c r="H3" s="26" t="n"/>
+      <c r="I3" s="26" t="n"/>
+    </row>
+    <row r="4" ht="21.75" customFormat="1" customHeight="1" s="72">
+      <c r="A4" s="64" t="n"/>
+      <c r="B4" s="71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Create a folder named &lt;HOTEN_MSSV_NHOM&gt; to save the files after finishing the tasks, </t>
+        </is>
+      </c>
+      <c r="C4" s="66" t="n"/>
+      <c r="D4" s="71" t="n"/>
+      <c r="E4" s="71" t="n"/>
+      <c r="F4" s="71" t="n"/>
+      <c r="G4" s="71" t="n"/>
+      <c r="H4" s="71" t="n"/>
+      <c r="I4" s="71" t="n"/>
+    </row>
+    <row r="5" customFormat="1" s="72">
+      <c r="B5" s="72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                 sau khi làm xong BT, nén thư mục lại và chuyển lên hệ thống elearning.</t>
+        </is>
+      </c>
+      <c r="C5" s="71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">archive the folder to a rar file and upload the archived file to the Elearning site. </t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="26" t="n"/>
+      <c r="B6" s="25" t="inlineStr">
+        <is>
+          <t>Only perform the tasks on this sheet. Other sheets are for support.</t>
+        </is>
+      </c>
+      <c r="C6" s="26" t="n"/>
+      <c r="D6" s="26" t="n"/>
+      <c r="E6" s="26" t="n"/>
+      <c r="F6" s="26" t="n"/>
+      <c r="G6" s="26" t="n"/>
+      <c r="H6" s="26" t="n"/>
+      <c r="I6" s="26" t="n"/>
+    </row>
+    <row r="7" ht="15.75" customFormat="1" customHeight="1" s="60">
+      <c r="B7" s="26" t="n"/>
+      <c r="C7" s="30" t="n"/>
+      <c r="K7" s="61" t="n"/>
+      <c r="L7" s="61" t="n"/>
+      <c r="M7" s="61" t="n"/>
+      <c r="N7" s="61" t="n"/>
+      <c r="O7" s="61" t="n"/>
+      <c r="P7" s="61" t="n"/>
+    </row>
+    <row r="8" customFormat="1" s="76">
+      <c r="A8" s="73" t="inlineStr">
+        <is>
+          <t>I.-</t>
+        </is>
+      </c>
+      <c r="B8" s="77" t="inlineStr">
+        <is>
+          <t>In the bai 1 worksheet, perform the following tasks:</t>
+        </is>
+      </c>
+      <c r="C8" s="75" t="n"/>
+      <c r="D8" s="75" t="n"/>
+      <c r="E8" s="75" t="n"/>
+      <c r="F8" s="75" t="n"/>
+      <c r="G8" s="75" t="n"/>
+      <c r="H8" s="75" t="n"/>
+      <c r="I8" s="79" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="70" t="n"/>
+      <c r="B9" s="70" t="inlineStr">
+        <is>
+          <t>1/</t>
+        </is>
+      </c>
+      <c r="C9" s="71" t="inlineStr">
+        <is>
+          <t>Fill series to the STT column (A4:A10 and K4:K10).</t>
+        </is>
+      </c>
+      <c r="D9" s="71" t="n"/>
+      <c r="E9" s="71" t="n"/>
+      <c r="F9" s="71" t="n"/>
+      <c r="G9" s="71" t="n"/>
+      <c r="H9" s="71" t="n"/>
+      <c r="I9" s="71" t="n"/>
+      <c r="J9" s="26" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="70" t="n"/>
+      <c r="B10" s="70" t="inlineStr">
+        <is>
+          <t>2/</t>
+        </is>
+      </c>
+      <c r="C10" s="71" t="inlineStr">
+        <is>
+          <t>Trị giá = Số lượng * Đơn giá.</t>
+        </is>
+      </c>
+      <c r="D10" s="71" t="n"/>
+      <c r="E10" s="71" t="n"/>
+      <c r="F10" s="71" t="n"/>
+      <c r="G10" s="71" t="n"/>
+      <c r="H10" s="71" t="n"/>
+      <c r="I10" s="71" t="n"/>
+      <c r="J10" s="26" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="70" t="n"/>
+      <c r="B11" s="70" t="inlineStr">
+        <is>
+          <t>3/</t>
+        </is>
+      </c>
+      <c r="C11" s="71" t="inlineStr">
+        <is>
+          <t>Thuế = Trị giá * 5%.</t>
+        </is>
+      </c>
+      <c r="D11" s="71" t="n"/>
+      <c r="E11" s="71" t="n"/>
+      <c r="F11" s="71" t="n"/>
+      <c r="G11" s="71" t="n"/>
+      <c r="H11" s="71" t="n"/>
+      <c r="I11" s="71" t="n"/>
+      <c r="J11" s="26" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="70" t="n"/>
+      <c r="B12" s="70" t="inlineStr">
+        <is>
+          <t>4/</t>
+        </is>
+      </c>
+      <c r="C12" s="71" t="inlineStr">
+        <is>
+          <t>Cước chuyên chở = Số lượng * 1500.</t>
+        </is>
+      </c>
+      <c r="D12" s="71" t="n"/>
+      <c r="E12" s="71" t="n"/>
+      <c r="F12" s="71" t="n"/>
+      <c r="G12" s="71" t="n"/>
+      <c r="H12" s="71" t="n"/>
+      <c r="I12" s="71" t="n"/>
+      <c r="J12" s="26" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="70" t="n"/>
+      <c r="B13" s="70" t="inlineStr">
+        <is>
+          <t>5/</t>
+        </is>
+      </c>
+      <c r="C13" s="71" t="inlineStr">
+        <is>
+          <t>Cộng USD = Trị giá + Thuế + Cước chuyên chở.</t>
+        </is>
+      </c>
+      <c r="D13" s="71" t="n"/>
+      <c r="E13" s="71" t="n"/>
+      <c r="F13" s="71" t="n"/>
+      <c r="G13" s="71" t="n"/>
+      <c r="H13" s="71" t="n"/>
+      <c r="I13" s="71" t="n"/>
+      <c r="J13" s="26" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="70" t="n"/>
+      <c r="B14" s="70" t="inlineStr">
+        <is>
+          <t>6/</t>
+        </is>
+      </c>
+      <c r="C14" s="71" t="inlineStr">
+        <is>
+          <t>Cộng VNĐ are converted based on columns Cộng USD and Tỉ giá.</t>
+        </is>
+      </c>
+      <c r="D14" s="71" t="n"/>
+      <c r="E14" s="71" t="n"/>
+      <c r="F14" s="71" t="n"/>
+      <c r="G14" s="71" t="n"/>
+      <c r="H14" s="71" t="n"/>
+      <c r="I14" s="71" t="n"/>
+      <c r="J14" s="26" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="70" t="n"/>
+      <c r="B15" s="70" t="n"/>
+      <c r="C15" s="71" t="inlineStr">
+        <is>
+          <t>Cộng VNĐ = Cộng USD * Tỉ giá.</t>
+        </is>
+      </c>
+      <c r="D15" s="71" t="n"/>
+      <c r="E15" s="71" t="n"/>
+      <c r="F15" s="71" t="n"/>
+      <c r="G15" s="71" t="n"/>
+      <c r="H15" s="71" t="n"/>
+      <c r="I15" s="71" t="n"/>
+      <c r="J15" s="26" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="70" t="n"/>
+      <c r="B16" s="70" t="inlineStr">
+        <is>
+          <t>7/</t>
+        </is>
+      </c>
+      <c r="C16" s="71" t="inlineStr">
+        <is>
+          <t>The January profit of each item is calculated by adding its January profit in 2014, 2015 and 2016 together.</t>
+        </is>
+      </c>
+      <c r="D16" s="71" t="n"/>
+      <c r="E16" s="71" t="n"/>
+      <c r="F16" s="71" t="n"/>
+      <c r="G16" s="71" t="n"/>
+      <c r="H16" s="71" t="n"/>
+      <c r="I16" s="71" t="n"/>
+      <c r="J16" s="26" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="70" t="n"/>
+      <c r="B17" s="70" t="inlineStr">
+        <is>
+          <t>8/</t>
+        </is>
+      </c>
+      <c r="C17" s="71" t="inlineStr">
+        <is>
+          <t>Copy the formula so that it can show the total profit of each item in each month of the whole 3 years.</t>
+        </is>
+      </c>
+      <c r="D17" s="71" t="n"/>
+      <c r="E17" s="71" t="n"/>
+      <c r="F17" s="71" t="n"/>
+      <c r="G17" s="71" t="n"/>
+      <c r="H17" s="71" t="n"/>
+      <c r="I17" s="71" t="n"/>
+      <c r="J17" s="26" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="70" t="n"/>
+      <c r="B18" s="70" t="inlineStr">
+        <is>
+          <t>9/</t>
+        </is>
+      </c>
+      <c r="C18" s="71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Calculate the total profit of all items in all months. </t>
+        </is>
+      </c>
+      <c r="D18" s="71" t="n"/>
+      <c r="E18" s="71" t="n"/>
+      <c r="F18" s="71" t="n"/>
+      <c r="G18" s="71" t="n"/>
+      <c r="H18" s="71" t="n"/>
+      <c r="I18" s="71" t="n"/>
+      <c r="J18" s="26" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="70" t="n"/>
+      <c r="B19" s="70" t="inlineStr">
+        <is>
+          <t>10/</t>
+        </is>
+      </c>
+      <c r="C19" s="71" t="inlineStr">
+        <is>
+          <t>Calculate the biggest lost value of Tháng 1.</t>
+        </is>
+      </c>
+      <c r="D19" s="71" t="n"/>
+      <c r="E19" s="71" t="n"/>
+      <c r="F19" s="71" t="n"/>
+      <c r="G19" s="71" t="n"/>
+      <c r="H19" s="71" t="n"/>
+      <c r="I19" s="71" t="n"/>
+      <c r="J19" s="26" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="70" t="n"/>
+      <c r="B20" s="70" t="inlineStr">
+        <is>
+          <t>11/</t>
+        </is>
+      </c>
+      <c r="C20" s="71" t="inlineStr">
+        <is>
+          <t>Calculate the biggest profit value of Tháng 3.</t>
+        </is>
+      </c>
+      <c r="D20" s="71" t="n"/>
+      <c r="E20" s="71" t="n"/>
+      <c r="F20" s="71" t="n"/>
+      <c r="G20" s="71" t="n"/>
+      <c r="H20" s="71" t="n"/>
+      <c r="I20" s="71" t="n"/>
+      <c r="J20" s="26" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="70" t="n"/>
+      <c r="B21" s="70" t="inlineStr">
+        <is>
+          <t>12/</t>
+        </is>
+      </c>
+      <c r="C21" s="71" t="inlineStr">
+        <is>
+          <t>Calculate the average profit value of Tháng 5.</t>
+        </is>
+      </c>
+      <c r="D21" s="71" t="n"/>
+      <c r="E21" s="71" t="n"/>
+      <c r="F21" s="71" t="n"/>
+      <c r="G21" s="71" t="n"/>
+      <c r="H21" s="71" t="n"/>
+      <c r="I21" s="71" t="n"/>
+      <c r="J21" s="26" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="70" t="n"/>
+      <c r="B22" s="70" t="inlineStr">
+        <is>
+          <t>13/</t>
+        </is>
+      </c>
+      <c r="C22" s="71" t="inlineStr">
+        <is>
+          <t>Save the file.</t>
+        </is>
+      </c>
+      <c r="D22" s="72" t="n"/>
+      <c r="E22" s="71" t="n"/>
+      <c r="F22" s="71" t="n"/>
+      <c r="G22" s="71" t="n"/>
+      <c r="H22" s="71" t="n"/>
+      <c r="I22" s="71" t="n"/>
+      <c r="J22" s="26" t="n"/>
+    </row>
+    <row r="23" customFormat="1" s="76">
+      <c r="A23" s="73" t="inlineStr">
+        <is>
+          <t>II.-</t>
+        </is>
+      </c>
+      <c r="B23" s="77" t="inlineStr">
+        <is>
+          <t>In the 2016 worksheet, perform the following tasks:</t>
+        </is>
+      </c>
+      <c r="C23" s="75" t="n"/>
+      <c r="D23" s="75" t="n"/>
+      <c r="E23" s="75" t="n"/>
+      <c r="F23" s="75" t="n"/>
+      <c r="G23" s="75" t="n"/>
+      <c r="H23" s="75" t="n"/>
+      <c r="I23" s="75" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="70" t="n"/>
+      <c r="B24" s="70" t="inlineStr">
+        <is>
+          <t>1/</t>
+        </is>
+      </c>
+      <c r="C24" s="72" t="inlineStr">
+        <is>
+          <t>Name the C3:H9 range DATA.</t>
+        </is>
+      </c>
+      <c r="D24" s="71" t="n"/>
+      <c r="E24" s="71" t="n"/>
+      <c r="F24" s="71" t="n"/>
+      <c r="G24" s="71" t="n"/>
+      <c r="H24" s="71" t="n"/>
+      <c r="I24" s="71" t="n"/>
+      <c r="J24" s="26" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="70" t="n"/>
+      <c r="B25" s="70" t="inlineStr">
+        <is>
+          <t>2/</t>
+        </is>
+      </c>
+      <c r="C25" s="72" t="inlineStr">
+        <is>
+          <t>Use the DATA range name, calculate the total profit of all items in all months.</t>
+        </is>
+      </c>
+      <c r="D25" s="71" t="n"/>
+      <c r="E25" s="71" t="n"/>
+      <c r="F25" s="71" t="n"/>
+      <c r="G25" s="71" t="n"/>
+      <c r="H25" s="71" t="n"/>
+      <c r="I25" s="71" t="n"/>
+      <c r="J25" s="26" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="70" t="n"/>
+      <c r="B26" s="70" t="inlineStr">
+        <is>
+          <t>3/</t>
+        </is>
+      </c>
+      <c r="C26" s="72" t="inlineStr">
+        <is>
+          <t>Use the DATA range name, calculate the max profit of all items in all months.</t>
+        </is>
+      </c>
+      <c r="D26" s="71" t="n"/>
+      <c r="E26" s="71" t="n"/>
+      <c r="F26" s="71" t="n"/>
+      <c r="G26" s="71" t="n"/>
+      <c r="H26" s="71" t="n"/>
+      <c r="I26" s="71" t="n"/>
+      <c r="J26" s="26" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="70" t="n"/>
+      <c r="B27" s="70" t="inlineStr">
+        <is>
+          <t>4/</t>
+        </is>
+      </c>
+      <c r="C27" s="72" t="inlineStr">
+        <is>
+          <t>Use the DATA range name, calculate the average profit of all items in all months.</t>
+        </is>
+      </c>
+      <c r="D27" s="71" t="n"/>
+      <c r="E27" s="71" t="n"/>
+      <c r="F27" s="71" t="n"/>
+      <c r="G27" s="71" t="n"/>
+      <c r="H27" s="71" t="n"/>
+      <c r="I27" s="71" t="n"/>
+      <c r="J27" s="26" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="72" t="n"/>
+      <c r="B28" s="70" t="inlineStr">
+        <is>
+          <t>5/</t>
+        </is>
+      </c>
+      <c r="C28" s="72" t="inlineStr">
+        <is>
+          <t>Display formulas instead of the values of formulas.</t>
+        </is>
+      </c>
+      <c r="D28" s="72" t="n"/>
+      <c r="E28" s="72" t="n"/>
+      <c r="F28" s="72" t="n"/>
+      <c r="G28" s="72" t="n"/>
+      <c r="H28" s="72" t="n"/>
+      <c r="I28" s="72" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="72" t="n"/>
+      <c r="B29" s="70" t="inlineStr">
+        <is>
+          <t>6/</t>
+        </is>
+      </c>
+      <c r="C29" s="71" t="inlineStr">
+        <is>
+          <t>Save the file.</t>
+        </is>
+      </c>
+      <c r="D29" s="72" t="n"/>
+      <c r="E29" s="72" t="n"/>
+      <c r="F29" s="72" t="n"/>
+      <c r="G29" s="72" t="n"/>
+      <c r="H29" s="72" t="n"/>
+      <c r="I29" s="72" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="72" t="n"/>
+      <c r="B30" s="72" t="n"/>
+      <c r="C30" s="72" t="n"/>
+      <c r="D30" s="72" t="n"/>
+      <c r="E30" s="72" t="n"/>
+      <c r="F30" s="72" t="n"/>
+      <c r="G30" s="72" t="n"/>
+      <c r="H30" s="72" t="n"/>
+      <c r="I30" s="72" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="72" t="n"/>
+      <c r="B31" s="72" t="n"/>
+      <c r="C31" s="72" t="n"/>
+      <c r="D31" s="72" t="n"/>
+      <c r="E31" s="72" t="n"/>
+      <c r="F31" s="72" t="n"/>
+      <c r="G31" s="72" t="n"/>
+      <c r="H31" s="72" t="n"/>
+      <c r="I31" s="72" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2145,7 +3300,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2503,7 +3658,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2762,7 +3917,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Restore original banner shapes on the requirement sheets of bài6 and bài7
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HiyVPr15dFfxwtDW3Tiv76
</commit_message>
<xml_diff>
--- a/excel_bai_tap/TranGiaHy_11a2_bài6.xlsx
+++ b/excel_bai_tap/TranGiaHy_11a2_bài6.xlsx
@@ -628,123 +628,585 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <twoCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>465896</colOff>
-      <row>0</row>
-      <rowOff>0</rowOff>
-    </from>
-    <to>
-      <col>12</col>
-      <colOff>55079</colOff>
-      <row>3</row>
-      <rowOff>5763</rowOff>
-    </to>
-    <grpSp>
-      <nvGrpSpPr>
-        <cNvPr id="3" name="Group 2"/>
-        <cNvGrpSpPr/>
-      </nvGrpSpPr>
-      <grpSpPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0">
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>465896</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>55079</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>5763</xdr:rowOff>
+    </xdr:to>
+    <xdr:grpSp>
+      <xdr:nvGrpSpPr>
+        <xdr:cNvPr id="3" name="Group 2"/>
+        <xdr:cNvGrpSpPr/>
+      </xdr:nvGrpSpPr>
+      <xdr:grpSpPr>
+        <a:xfrm>
           <a:off x="1087092" y="0"/>
           <a:ext cx="5718313" cy="651806"/>
           <a:chOff x="10002807" y="3305175"/>
           <a:chExt cx="9771093" cy="832807"/>
         </a:xfrm>
-      </grpSpPr>
-      <pic>
-        <nvPicPr>
-          <cNvPr id="7" name="Picture 6"/>
-          <cNvPicPr>
-            <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-          </cNvPicPr>
-        </nvPicPr>
-        <blipFill>
-          <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
-          <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      </xdr:grpSpPr>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="4" name="Rounded Rectangle 3"/>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="10020300" y="3333750"/>
+            <a:ext cx="9753600" cy="781050"/>
+          </a:xfrm>
+          <a:prstGeom prst="roundRect">
+            <a:avLst/>
+          </a:prstGeom>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="2">
+            <a:schemeClr val="accent6"/>
+          </a:lnRef>
+          <a:fillRef idx="1">
+            <a:schemeClr val="lt1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent6"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="dk1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="l"/>
+            <a:endParaRPr lang="en-US" sz="1100"/>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:pic>
+        <xdr:nvPicPr>
+          <xdr:cNvPr id="5" name="Picture 4"/>
+          <xdr:cNvPicPr>
+            <a:picLocks noChangeAspect="1"/>
+          </xdr:cNvPicPr>
+        </xdr:nvPicPr>
+        <xdr:blipFill>
+          <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
+            <a:extLst>
+              <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+                <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+              </a:ext>
+            </a:extLst>
+          </a:blip>
+          <a:stretch>
             <a:fillRect/>
           </a:stretch>
-        </blipFill>
-        <spPr>
-          <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        </xdr:blipFill>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="18487371" y="3422438"/>
+            <a:ext cx="1055163" cy="715544"/>
+          </a:xfrm>
+          <a:prstGeom prst="ellipse">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst>
+            <a:softEdge rad="112500"/>
+          </a:effectLst>
+        </xdr:spPr>
+      </xdr:pic>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="6" name="Rectangle 5"/>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="10002807" y="3305175"/>
+            <a:ext cx="9744852" cy="736721"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:noFill/>
+        </xdr:spPr>
+        <xdr:txBody>
+          <a:bodyPr wrap="square" lIns="91440" tIns="45720" rIns="91440" bIns="45720">
+            <a:spAutoFit/>
+            <a:scene3d>
+              <a:camera prst="orthographicFront"/>
+              <a:lightRig rig="flat" dir="tl">
+                <a:rot lat="0" lon="0" rev="6600000"/>
+              </a:lightRig>
+            </a:scene3d>
+            <a:sp3d extrusionH="25400" contourW="8890">
+              <a:bevelT w="38100" h="31750"/>
+              <a:contourClr>
+                <a:schemeClr val="accent2">
+                  <a:shade val="75000"/>
+                </a:schemeClr>
+              </a:contourClr>
+            </a:sp3d>
+          </a:bodyPr>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="ctr"/>
+            <a:r>
+              <a:rPr lang="en-US" sz="3000" b="1" cap="none" spc="0">
+                <a:ln w="11430"/>
+                <a:gradFill>
+                  <a:gsLst>
+                    <a:gs pos="0">
+                      <a:schemeClr val="accent2">
+                        <a:tint val="70000"/>
+                        <a:satMod val="245000"/>
+                      </a:schemeClr>
+                    </a:gs>
+                    <a:gs pos="75000">
+                      <a:schemeClr val="accent2">
+                        <a:tint val="90000"/>
+                        <a:shade val="60000"/>
+                        <a:satMod val="240000"/>
+                      </a:schemeClr>
+                    </a:gs>
+                    <a:gs pos="100000">
+                      <a:schemeClr val="accent2">
+                        <a:tint val="100000"/>
+                        <a:shade val="50000"/>
+                        <a:satMod val="240000"/>
+                      </a:schemeClr>
+                    </a:gs>
+                  </a:gsLst>
+                  <a:lin ang="5400000"/>
+                </a:gradFill>
+                <a:effectLst>
+                  <a:outerShdw blurRad="50800" dist="39000" dir="5460000" algn="tl">
+                    <a:srgbClr val="000000">
+                      <a:alpha val="38000"/>
+                    </a:srgbClr>
+                  </a:outerShdw>
+                </a:effectLst>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:rPr>
+              <a:t>  BÀI</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" sz="3000" b="1" cap="none" spc="0" baseline="0">
+                <a:ln w="11430"/>
+                <a:gradFill>
+                  <a:gsLst>
+                    <a:gs pos="0">
+                      <a:schemeClr val="accent2">
+                        <a:tint val="70000"/>
+                        <a:satMod val="245000"/>
+                      </a:schemeClr>
+                    </a:gs>
+                    <a:gs pos="75000">
+                      <a:schemeClr val="accent2">
+                        <a:tint val="90000"/>
+                        <a:shade val="60000"/>
+                        <a:satMod val="240000"/>
+                      </a:schemeClr>
+                    </a:gs>
+                    <a:gs pos="100000">
+                      <a:schemeClr val="accent2">
+                        <a:tint val="100000"/>
+                        <a:shade val="50000"/>
+                        <a:satMod val="240000"/>
+                      </a:schemeClr>
+                    </a:gs>
+                  </a:gsLst>
+                  <a:lin ang="5400000"/>
+                </a:gradFill>
+                <a:effectLst>
+                  <a:outerShdw blurRad="50800" dist="39000" dir="5460000" algn="tl">
+                    <a:srgbClr val="000000">
+                      <a:alpha val="38000"/>
+                    </a:srgbClr>
+                  </a:outerShdw>
+                </a:effectLst>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:rPr>
+              <a:t> TẬP VỀ NHÀ TUẦN 7</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-US" sz="3000" b="1" cap="none" spc="0">
+              <a:ln w="11430"/>
+              <a:gradFill>
+                <a:gsLst>
+                  <a:gs pos="0">
+                    <a:schemeClr val="accent2">
+                      <a:tint val="70000"/>
+                      <a:satMod val="245000"/>
+                    </a:schemeClr>
+                  </a:gs>
+                  <a:gs pos="75000">
+                    <a:schemeClr val="accent2">
+                      <a:tint val="90000"/>
+                      <a:shade val="60000"/>
+                      <a:satMod val="240000"/>
+                    </a:schemeClr>
+                  </a:gs>
+                  <a:gs pos="100000">
+                    <a:schemeClr val="accent2">
+                      <a:tint val="100000"/>
+                      <a:shade val="50000"/>
+                      <a:satMod val="240000"/>
+                    </a:schemeClr>
+                  </a:gs>
+                </a:gsLst>
+                <a:lin ang="5400000"/>
+              </a:gradFill>
+              <a:effectLst>
+                <a:outerShdw blurRad="50800" dist="39000" dir="5460000" algn="tl">
+                  <a:srgbClr val="000000">
+                    <a:alpha val="38000"/>
+                  </a:srgbClr>
+                </a:outerShdw>
+              </a:effectLst>
+            </a:endParaRPr>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:pic>
+        <xdr:nvPicPr>
+          <xdr:cNvPr id="7" name="Picture 6"/>
+          <xdr:cNvPicPr>
+            <a:picLocks noChangeAspect="1"/>
+          </xdr:cNvPicPr>
+        </xdr:nvPicPr>
+        <xdr:blipFill>
+          <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print">
+            <a:extLst>
+              <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+                <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+              </a:ext>
+            </a:extLst>
+          </a:blip>
+          <a:stretch>
+            <a:fillRect/>
+          </a:stretch>
+        </xdr:blipFill>
+        <xdr:spPr>
+          <a:xfrm>
             <a:off x="10358294" y="3459262"/>
             <a:ext cx="1123949" cy="621523"/>
           </a:xfrm>
-          <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-            <avLst/>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
           </a:prstGeom>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-            <a:prstDash val="solid"/>
-          </a:ln>
-        </spPr>
-      </pic>
-    </grpSp>
-    <clientData/>
-  </twoCellAnchor>
-</wsDr>
+        </xdr:spPr>
+      </xdr:pic>
+    </xdr:grpSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <twoCellAnchor>
-    <from>
-      <col>4</col>
-      <colOff>143511</colOff>
-      <row>0</row>
-      <rowOff>0</rowOff>
-    </from>
-    <to>
-      <col>13</col>
-      <colOff>343743</colOff>
-      <row>2</row>
-      <rowOff>184462</rowOff>
-    </to>
-    <grpSp>
-      <nvGrpSpPr>
-        <cNvPr id="2" name="Group 1"/>
-        <cNvGrpSpPr/>
-      </nvGrpSpPr>
-      <grpSpPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0">
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>143511</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>343743</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>184462</xdr:rowOff>
+    </xdr:to>
+    <xdr:grpSp>
+      <xdr:nvGrpSpPr>
+        <xdr:cNvPr id="2" name="Group 1"/>
+        <xdr:cNvGrpSpPr/>
+      </xdr:nvGrpSpPr>
+      <xdr:grpSpPr>
+        <a:xfrm>
           <a:off x="1970579" y="0"/>
           <a:ext cx="5655459" cy="634735"/>
           <a:chOff x="10002807" y="3305175"/>
           <a:chExt cx="9744851" cy="809625"/>
         </a:xfrm>
-      </grpSpPr>
-      <pic>
-        <nvPicPr>
-          <cNvPr id="6" name="Picture 5"/>
-          <cNvPicPr>
-            <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-          </cNvPicPr>
-        </nvPicPr>
-        <blipFill>
-          <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
-          <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      </xdr:grpSpPr>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="3" name="Rounded Rectangle 2"/>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="10020299" y="3333750"/>
+            <a:ext cx="9036259" cy="781050"/>
+          </a:xfrm>
+          <a:prstGeom prst="roundRect">
+            <a:avLst/>
+          </a:prstGeom>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="2">
+            <a:schemeClr val="accent6"/>
+          </a:lnRef>
+          <a:fillRef idx="1">
+            <a:schemeClr val="lt1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent6"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="dk1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="l"/>
+            <a:endParaRPr lang="en-US" sz="1100"/>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:pic>
+        <xdr:nvPicPr>
+          <xdr:cNvPr id="4" name="Picture 3"/>
+          <xdr:cNvPicPr>
+            <a:picLocks noChangeAspect="1"/>
+          </xdr:cNvPicPr>
+        </xdr:nvPicPr>
+        <xdr:blipFill>
+          <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
+            <a:extLst>
+              <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+                <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+              </a:ext>
+            </a:extLst>
+          </a:blip>
+          <a:stretch>
             <a:fillRect/>
           </a:stretch>
-        </blipFill>
-        <spPr>
-          <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        </xdr:blipFill>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="17654102" y="3378039"/>
+            <a:ext cx="1055162" cy="715544"/>
+          </a:xfrm>
+          <a:prstGeom prst="ellipse">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst>
+            <a:softEdge rad="112500"/>
+          </a:effectLst>
+        </xdr:spPr>
+      </xdr:pic>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="5" name="Rectangle 4"/>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="10002807" y="3305175"/>
+            <a:ext cx="9744851" cy="681050"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:noFill/>
+        </xdr:spPr>
+        <xdr:txBody>
+          <a:bodyPr wrap="square" lIns="91440" tIns="45720" rIns="91440" bIns="45720">
+            <a:spAutoFit/>
+            <a:scene3d>
+              <a:camera prst="orthographicFront"/>
+              <a:lightRig rig="flat" dir="tl">
+                <a:rot lat="0" lon="0" rev="6600000"/>
+              </a:lightRig>
+            </a:scene3d>
+            <a:sp3d extrusionH="25400" contourW="8890">
+              <a:bevelT w="38100" h="31750"/>
+              <a:contourClr>
+                <a:schemeClr val="accent2">
+                  <a:shade val="75000"/>
+                </a:schemeClr>
+              </a:contourClr>
+            </a:sp3d>
+          </a:bodyPr>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="ctr"/>
+            <a:r>
+              <a:rPr lang="en-US" sz="3000" b="1" cap="none" spc="0">
+                <a:ln w="11430"/>
+                <a:gradFill>
+                  <a:gsLst>
+                    <a:gs pos="0">
+                      <a:schemeClr val="accent2">
+                        <a:tint val="70000"/>
+                        <a:satMod val="245000"/>
+                      </a:schemeClr>
+                    </a:gs>
+                    <a:gs pos="75000">
+                      <a:schemeClr val="accent2">
+                        <a:tint val="90000"/>
+                        <a:shade val="60000"/>
+                        <a:satMod val="240000"/>
+                      </a:schemeClr>
+                    </a:gs>
+                    <a:gs pos="100000">
+                      <a:schemeClr val="accent2">
+                        <a:tint val="100000"/>
+                        <a:shade val="50000"/>
+                        <a:satMod val="240000"/>
+                      </a:schemeClr>
+                    </a:gs>
+                  </a:gsLst>
+                  <a:lin ang="5400000"/>
+                </a:gradFill>
+                <a:effectLst>
+                  <a:outerShdw blurRad="50800" dist="39000" dir="5460000" algn="tl">
+                    <a:srgbClr val="000000">
+                      <a:alpha val="38000"/>
+                    </a:srgbClr>
+                  </a:outerShdw>
+                </a:effectLst>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:rPr>
+              <a:t>Homework Week</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" sz="3000" b="1" cap="none" spc="0" baseline="0">
+                <a:ln w="11430"/>
+                <a:gradFill>
+                  <a:gsLst>
+                    <a:gs pos="0">
+                      <a:schemeClr val="accent2">
+                        <a:tint val="70000"/>
+                        <a:satMod val="245000"/>
+                      </a:schemeClr>
+                    </a:gs>
+                    <a:gs pos="75000">
+                      <a:schemeClr val="accent2">
+                        <a:tint val="90000"/>
+                        <a:shade val="60000"/>
+                        <a:satMod val="240000"/>
+                      </a:schemeClr>
+                    </a:gs>
+                    <a:gs pos="100000">
+                      <a:schemeClr val="accent2">
+                        <a:tint val="100000"/>
+                        <a:shade val="50000"/>
+                        <a:satMod val="240000"/>
+                      </a:schemeClr>
+                    </a:gs>
+                  </a:gsLst>
+                  <a:lin ang="5400000"/>
+                </a:gradFill>
+                <a:effectLst>
+                  <a:outerShdw blurRad="50800" dist="39000" dir="5460000" algn="tl">
+                    <a:srgbClr val="000000">
+                      <a:alpha val="38000"/>
+                    </a:srgbClr>
+                  </a:outerShdw>
+                </a:effectLst>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:rPr>
+              <a:t> 7</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-US" sz="3000" b="1" cap="none" spc="0">
+              <a:ln w="11430"/>
+              <a:gradFill>
+                <a:gsLst>
+                  <a:gs pos="0">
+                    <a:schemeClr val="accent2">
+                      <a:tint val="70000"/>
+                      <a:satMod val="245000"/>
+                    </a:schemeClr>
+                  </a:gs>
+                  <a:gs pos="75000">
+                    <a:schemeClr val="accent2">
+                      <a:tint val="90000"/>
+                      <a:shade val="60000"/>
+                      <a:satMod val="240000"/>
+                    </a:schemeClr>
+                  </a:gs>
+                  <a:gs pos="100000">
+                    <a:schemeClr val="accent2">
+                      <a:tint val="100000"/>
+                      <a:shade val="50000"/>
+                      <a:satMod val="240000"/>
+                    </a:schemeClr>
+                  </a:gs>
+                </a:gsLst>
+                <a:lin ang="5400000"/>
+              </a:gradFill>
+              <a:effectLst>
+                <a:outerShdw blurRad="50800" dist="39000" dir="5460000" algn="tl">
+                  <a:srgbClr val="000000">
+                    <a:alpha val="38000"/>
+                  </a:srgbClr>
+                </a:outerShdw>
+              </a:effectLst>
+            </a:endParaRPr>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:pic>
+        <xdr:nvPicPr>
+          <xdr:cNvPr id="6" name="Picture 5"/>
+          <xdr:cNvPicPr>
+            <a:picLocks noChangeAspect="1"/>
+          </xdr:cNvPicPr>
+        </xdr:nvPicPr>
+        <xdr:blipFill>
+          <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print">
+            <a:extLst>
+              <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+                <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+              </a:ext>
+            </a:extLst>
+          </a:blip>
+          <a:stretch>
+            <a:fillRect/>
+          </a:stretch>
+        </xdr:blipFill>
+        <xdr:spPr>
+          <a:xfrm>
             <a:off x="10358292" y="3459263"/>
             <a:ext cx="1442521" cy="621523"/>
           </a:xfrm>
-          <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-            <avLst/>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
           </a:prstGeom>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-            <a:prstDash val="solid"/>
-          </a:ln>
-        </spPr>
-      </pic>
-    </grpSp>
-    <clientData/>
-  </twoCellAnchor>
-</wsDr>
+        </xdr:spPr>
+      </xdr:pic>
+    </xdr:grpSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
Fix bài6/bài7: keep rich text on requirement sheets, unrotate D3/E3 headers
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HiyVPr15dFfxwtDW3Tiv76
</commit_message>
<xml_diff>
--- a/excel_bai_tap/TranGiaHy_11a2_bài6.xlsx
+++ b/excel_bai_tap/TranGiaHy_11a2_bài6.xlsx
@@ -1538,7 +1538,26 @@
       <c r="A4" s="29" t="n"/>
       <c r="B4" s="26" t="inlineStr">
         <is>
-          <t>Tạo thư mục &lt;HOTEN_MSSV&gt; để lưu các tập tin, nén thư mục này và nộp lên hệ thống Elearning</t>
+          <r>
+            <t xml:space="preserve">Tạo thư mục </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <b val="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>&lt;HOTEN_MSSV&gt;</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve"> để lưu các tập tin, nén thư mục này và nộp lên hệ thống Elearning</t>
+          </r>
         </is>
       </c>
       <c r="C4" s="26" t="n"/>
@@ -1553,7 +1572,30 @@
       <c r="A5" s="26" t="n"/>
       <c r="B5" s="25" t="inlineStr">
         <is>
-          <t>Chỉ thực hiện các yêu cầu trong trang tính này. Các trang tính khác dùng để hỗ trợ.</t>
+          <r>
+            <t xml:space="preserve">Chỉ thực hiện các yêu cầu trong trang tính này. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <b val="1"/>
+              <i val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Các trang tính khác dùng để hỗ trợ</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <i val="1"/>
+              <color rgb="FFFF0000"/>
+              <sz val="12"/>
+            </rPr>
+            <t>.</t>
+          </r>
         </is>
       </c>
       <c r="C5" s="26" t="n"/>
@@ -1572,7 +1614,30 @@
       </c>
       <c r="B6" s="77" t="inlineStr">
         <is>
-          <t>Trong trang tính bai 1 thực hiện các yêu cầu sau:</t>
+          <r>
+            <t xml:space="preserve">Trong trang tính </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <b val="1"/>
+              <i val="1"/>
+              <color rgb="FF0000FF"/>
+              <sz val="12"/>
+            </rPr>
+            <t>bai 1</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <i val="1"/>
+              <color rgb="FF0000FF"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve"> thực hiện các yêu cầu sau:</t>
+          </r>
         </is>
       </c>
       <c r="C6" s="75" t="n"/>
@@ -1592,7 +1657,60 @@
       </c>
       <c r="C7" s="26" t="inlineStr">
         <is>
-          <t>Điền số thứ tự cho các cột STT (A4:A10 và K4:K10) (autofill).</t>
+          <r>
+            <t xml:space="preserve">Điền số thứ tự cho các cột </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <b val="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>STT</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve"> (</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <b val="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>A4:A10</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve"> và </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <b val="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>K4:K10</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>) (autofill).</t>
+          </r>
         </is>
       </c>
       <c r="D7" s="26" t="n"/>
@@ -1612,7 +1730,57 @@
       </c>
       <c r="C8" s="26" t="inlineStr">
         <is>
-          <t>Trị giá = Số lượng * Đơn giá.</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <b val="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Trị giá</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve"> = </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <b val="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Số lượng</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve"> * </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <b val="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Đơn giá</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>.</t>
+          </r>
         </is>
       </c>
       <c r="D8" s="26" t="n"/>
@@ -1632,7 +1800,57 @@
       </c>
       <c r="C9" s="26" t="inlineStr">
         <is>
-          <t>Thuế = Trị giá * 5%.</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <b val="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Thuế</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve"> = </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <b val="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Trị giá</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve"> * </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <b val="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>5%</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>.</t>
+          </r>
         </is>
       </c>
       <c r="D9" s="26" t="n"/>
@@ -1652,7 +1870,57 @@
       </c>
       <c r="C10" s="26" t="inlineStr">
         <is>
-          <t>Cước chuyên chở = Số lượng * 1500.</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <b val="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Cước chuyên chở</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve"> = </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <b val="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Số lượng</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve"> * </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <b val="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>1500</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>.</t>
+          </r>
         </is>
       </c>
       <c r="D10" s="26" t="n"/>
@@ -1672,7 +1940,74 @@
       </c>
       <c r="C11" s="26" t="inlineStr">
         <is>
-          <t>Cộng USD = Trị giá + Thuế + Cước chuyên chở.</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <b val="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Cộng USD</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve"> =</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <b val="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve"> Trị giá</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve"> + </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <b val="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Thuế</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve"> + </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <b val="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Cước chuyên chở</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>.</t>
+          </r>
         </is>
       </c>
       <c r="D11" s="26" t="n"/>
@@ -1692,7 +2027,57 @@
       </c>
       <c r="C12" s="26" t="inlineStr">
         <is>
-          <t>Cộng VNĐ được qui đổi dựa vào cột Cộng USD và Tỉ giá..</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <b val="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Cộng VNĐ</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve"> được qui đổi dựa vào cột </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <b val="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Cộng USD</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve"> và </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <b val="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Tỉ giá.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>.</t>
+          </r>
         </is>
       </c>
       <c r="D12" s="26" t="n"/>
@@ -1712,7 +2097,26 @@
       </c>
       <c r="C13" s="26" t="inlineStr">
         <is>
-          <t>Tổng lợi nhuận THÁNG 1 của từng mặt hàng được tính bằng lợi nhuận tháng 1 trong các năm 2014, 2015 và 2016 của mặt hàng tương ứng.</t>
+          <r>
+            <t xml:space="preserve">Tổng lợi nhuận </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <b val="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>THÁNG 1</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve"> của từng mặt hàng được tính bằng lợi nhuận tháng 1 trong các năm 2014, 2015 và 2016 của mặt hàng tương ứng.</t>
+          </r>
         </is>
       </c>
       <c r="D13" s="26" t="n"/>
@@ -1772,7 +2176,26 @@
       </c>
       <c r="C16" s="26" t="inlineStr">
         <is>
-          <t>Xác định giá trị lỗ lớn nhất của tất cả các mặt hàng trong tháng 1.</t>
+          <r>
+            <t xml:space="preserve">Xác định giá trị lỗ lớn nhất của tất cả các mặt hàng trong tháng </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <b val="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>1</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>.</t>
+          </r>
         </is>
       </c>
       <c r="D16" s="26" t="n"/>
@@ -1792,7 +2215,26 @@
       </c>
       <c r="C17" s="26" t="inlineStr">
         <is>
-          <t>Xác định giá trị lãi lớn nhất của tất cả các mặt hàng trong tháng 3.</t>
+          <r>
+            <t xml:space="preserve">Xác định giá trị lãi lớn nhất của tất cả các mặt hàng trong tháng </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <b val="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>3</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>.</t>
+          </r>
         </is>
       </c>
       <c r="D17" s="26" t="n"/>
@@ -1812,7 +2254,26 @@
       </c>
       <c r="C18" s="26" t="inlineStr">
         <is>
-          <t>Xác định giá trị lợi nhuận trung bình của tất cả các mặt hàng trong tháng 5.</t>
+          <r>
+            <t xml:space="preserve">Xác định giá trị lợi nhuận trung bình của tất cả các mặt hàng trong tháng </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <b val="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>5</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>.</t>
+          </r>
         </is>
       </c>
       <c r="D18" s="26" t="n"/>
@@ -1851,7 +2312,30 @@
       </c>
       <c r="B20" s="77" t="inlineStr">
         <is>
-          <t>Trong trang tính 2016 thực hiện các yêu cầu sau:</t>
+          <r>
+            <t xml:space="preserve">Trong trang tính </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <b val="1"/>
+              <i val="1"/>
+              <color rgb="FF0000FF"/>
+              <sz val="12"/>
+            </rPr>
+            <t>2016</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <i val="1"/>
+              <color rgb="FF0000FF"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve"> thực hiện các yêu cầu sau:</t>
+          </r>
         </is>
       </c>
       <c r="C20" s="75" t="n"/>
@@ -1871,7 +2355,43 @@
       </c>
       <c r="C21" s="26" t="inlineStr">
         <is>
-          <t>Đặt tên cho khối ô C3:H9 là DATA.</t>
+          <r>
+            <t xml:space="preserve">Đặt tên cho khối ô </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <b val="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>C3:H9</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve"> là </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <b val="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>DATA</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>.</t>
+          </r>
         </is>
       </c>
       <c r="D21" s="26" t="n"/>
@@ -1891,7 +2411,26 @@
       </c>
       <c r="C22" s="26" t="inlineStr">
         <is>
-          <t>Sử dụng tên khối DATA, xác định tổng lợi nhuận của tất cả các mặt hàng trong tất cả các tháng.</t>
+          <r>
+            <t xml:space="preserve">Sử dụng tên khối </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <b val="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>DATA</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>, xác định tổng lợi nhuận của tất cả các mặt hàng trong tất cả các tháng.</t>
+          </r>
         </is>
       </c>
       <c r="D22" s="26" t="n"/>
@@ -1911,7 +2450,26 @@
       </c>
       <c r="C23" s="26" t="inlineStr">
         <is>
-          <t>Sử dụng tên khối DATA, xác định giá trị lợi nhuận lớn nhất của tất cả các mặt hàng trong tất cả các tháng</t>
+          <r>
+            <t xml:space="preserve">Sử dụng tên khối </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <b val="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>DATA</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>, xác định giá trị lợi nhuận lớn nhất của tất cả các mặt hàng trong tất cả các tháng</t>
+          </r>
         </is>
       </c>
       <c r="D23" s="26" t="n"/>
@@ -1931,7 +2489,26 @@
       </c>
       <c r="C24" s="26" t="inlineStr">
         <is>
-          <t>Sử dụng tên khối DATA, xác định giá trị lợi nhuận trung bình của tất cả các mặt hàng trong tất cả các tháng</t>
+          <r>
+            <t xml:space="preserve">Sử dụng tên khối </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <b val="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>DATA</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>, xác định giá trị lợi nhuận trung bình của tất cả các mặt hàng trong tất cả các tháng</t>
+          </r>
         </is>
       </c>
       <c r="D24" s="26" t="n"/>
@@ -2074,7 +2651,30 @@
       </c>
       <c r="B8" s="77" t="inlineStr">
         <is>
-          <t>In the bai 1 worksheet, perform the following tasks:</t>
+          <r>
+            <t xml:space="preserve">In the </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <b val="1"/>
+              <i val="1"/>
+              <color rgb="FF0000FF"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">bai 1 </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <i val="1"/>
+              <color rgb="FF0000FF"/>
+              <sz val="12"/>
+            </rPr>
+            <t>worksheet, perform the following tasks:</t>
+          </r>
         </is>
       </c>
       <c r="C8" s="75" t="n"/>
@@ -2094,7 +2694,66 @@
       </c>
       <c r="C9" s="71" t="inlineStr">
         <is>
-          <t>Fill series to the STT column (A4:A10 and K4:K10).</t>
+          <r>
+            <t xml:space="preserve">Fill series to the </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">STT </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>column (</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">A4:A10 </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">and </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>K4:K10</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>).</t>
+          </r>
         </is>
       </c>
       <c r="D9" s="71" t="n"/>
@@ -2114,7 +2773,63 @@
       </c>
       <c r="C10" s="71" t="inlineStr">
         <is>
-          <t>Trị giá = Số lượng * Đơn giá.</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Trị giá</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve"> = </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Số lượng</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve"> * </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Đơn giá</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>.</t>
+          </r>
         </is>
       </c>
       <c r="D10" s="71" t="n"/>
@@ -2134,7 +2849,63 @@
       </c>
       <c r="C11" s="71" t="inlineStr">
         <is>
-          <t>Thuế = Trị giá * 5%.</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Thuế</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve"> = </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Trị giá</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve"> * </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>5%</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>.</t>
+          </r>
         </is>
       </c>
       <c r="D11" s="71" t="n"/>
@@ -2154,7 +2925,63 @@
       </c>
       <c r="C12" s="71" t="inlineStr">
         <is>
-          <t>Cước chuyên chở = Số lượng * 1500.</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Cước chuyên chở</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve"> = </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Số lượng</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve"> * </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>1500</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>.</t>
+          </r>
         </is>
       </c>
       <c r="D12" s="71" t="n"/>
@@ -2174,7 +3001,82 @@
       </c>
       <c r="C13" s="71" t="inlineStr">
         <is>
-          <t>Cộng USD = Trị giá + Thuế + Cước chuyên chở.</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Cộng USD</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve"> =</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve"> Trị giá</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve"> + </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Thuế</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve"> + </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Cước chuyên chở</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>.</t>
+          </r>
         </is>
       </c>
       <c r="D13" s="71" t="n"/>
@@ -2194,7 +3096,63 @@
       </c>
       <c r="C14" s="71" t="inlineStr">
         <is>
-          <t>Cộng VNĐ are converted based on columns Cộng USD and Tỉ giá.</t>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Cộng VNĐ</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve"> are converted based on columns </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Cộng USD</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve"> and </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Tỉ giá</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>.</t>
+          </r>
         </is>
       </c>
       <c r="D14" s="71" t="n"/>
@@ -2230,7 +3188,104 @@
       </c>
       <c r="C16" s="71" t="inlineStr">
         <is>
-          <t>The January profit of each item is calculated by adding its January profit in 2014, 2015 and 2016 together.</t>
+          <r>
+            <t xml:space="preserve">The </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>January</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve"> profit of each item is calculated by adding its </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>January</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve"> profit in </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>2014,</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t> </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>2015</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve"> and </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>2016</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve"> together.</t>
+          </r>
         </is>
       </c>
       <c r="D16" s="71" t="n"/>
@@ -2290,7 +3345,28 @@
       </c>
       <c r="C19" s="71" t="inlineStr">
         <is>
-          <t>Calculate the biggest lost value of Tháng 1.</t>
+          <r>
+            <t xml:space="preserve">Calculate the biggest lost value of </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Tháng 1</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>.</t>
+          </r>
         </is>
       </c>
       <c r="D19" s="71" t="n"/>
@@ -2310,7 +3386,28 @@
       </c>
       <c r="C20" s="71" t="inlineStr">
         <is>
-          <t>Calculate the biggest profit value of Tháng 3.</t>
+          <r>
+            <t xml:space="preserve">Calculate the biggest profit value of </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Tháng 3</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>.</t>
+          </r>
         </is>
       </c>
       <c r="D20" s="71" t="n"/>
@@ -2330,7 +3427,28 @@
       </c>
       <c r="C21" s="71" t="inlineStr">
         <is>
-          <t>Calculate the average profit value of Tháng 5.</t>
+          <r>
+            <t xml:space="preserve">Calculate the average profit value of </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>Tháng 5</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>.</t>
+          </r>
         </is>
       </c>
       <c r="D21" s="71" t="n"/>
@@ -2369,7 +3487,30 @@
       </c>
       <c r="B23" s="77" t="inlineStr">
         <is>
-          <t>In the 2016 worksheet, perform the following tasks:</t>
+          <r>
+            <t xml:space="preserve">In the </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <b val="1"/>
+              <i val="1"/>
+              <color rgb="FF0000FF"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">2016 </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <i val="1"/>
+              <color rgb="FF0000FF"/>
+              <sz val="12"/>
+            </rPr>
+            <t>worksheet, perform the following tasks:</t>
+          </r>
         </is>
       </c>
       <c r="C23" s="75" t="n"/>
@@ -2389,7 +3530,38 @@
       </c>
       <c r="C24" s="72" t="inlineStr">
         <is>
-          <t>Name the C3:H9 range DATA.</t>
+          <r>
+            <t xml:space="preserve">Name the </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">C3:H9 </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">range </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>DATA.</t>
+          </r>
         </is>
       </c>
       <c r="D24" s="71" t="n"/>
@@ -2409,7 +3581,28 @@
       </c>
       <c r="C25" s="72" t="inlineStr">
         <is>
-          <t>Use the DATA range name, calculate the total profit of all items in all months.</t>
+          <r>
+            <t xml:space="preserve">Use the </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>DATA</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve"> range name, calculate the total profit of all items in all months.</t>
+          </r>
         </is>
       </c>
       <c r="D25" s="71" t="n"/>
@@ -2429,7 +3622,28 @@
       </c>
       <c r="C26" s="72" t="inlineStr">
         <is>
-          <t>Use the DATA range name, calculate the max profit of all items in all months.</t>
+          <r>
+            <t xml:space="preserve">Use the </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>DATA</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve"> range name, calculate the max profit of all items in all months.</t>
+          </r>
         </is>
       </c>
       <c r="D26" s="71" t="n"/>
@@ -2449,7 +3663,28 @@
       </c>
       <c r="C27" s="72" t="inlineStr">
         <is>
-          <t>Use the DATA range name, calculate the average profit of all items in all months.</t>
+          <r>
+            <t xml:space="preserve">Use the </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>DATA</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve"> range name, calculate the average profit of all items in all months.</t>
+          </r>
         </is>
       </c>
       <c r="D27" s="71" t="n"/>
@@ -2538,7 +3773,7 @@
   <cols>
     <col width="6" customWidth="1" style="26" min="1" max="1"/>
     <col width="7.5703125" customWidth="1" style="26" min="2" max="2"/>
-    <col width="10.28515625" customWidth="1" style="26" min="3" max="3"/>
+    <col width="12.5" customWidth="1" style="26" min="3" max="3"/>
     <col width="11.140625" customWidth="1" style="26" min="4" max="4"/>
     <col width="11.5703125" bestFit="1" customWidth="1" style="26" min="5" max="5"/>
     <col width="8.85546875" customWidth="1" style="26" min="6" max="6"/>
@@ -3045,13 +4280,13 @@
 LƯỢNG</t>
         </is>
       </c>
-      <c r="D3" s="48" t="inlineStr">
+      <c r="D3" s="47" t="inlineStr">
         <is>
           <t>ĐƠN
 GIÁ</t>
         </is>
       </c>
-      <c r="E3" s="49" t="inlineStr">
+      <c r="E3" s="47" t="inlineStr">
         <is>
           <t>TRỊ
 GIÁ</t>

</xml_diff>